<commit_message>
Configure 0.0.0.0 binding, health check endpoint, and Vercel routing
</commit_message>
<xml_diff>
--- a/blood_donors_50.xlsx
+++ b/blood_donors_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>demoperson011@gmail.com</t>
+          <t>ananyasingh23aiml@rnsit.ac.in</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         <v>140</v>
       </c>
       <c r="D3" t="n">
-        <v>916287672830</v>
+        <v>6287672830</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>O+</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>O+</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1625,6 +1625,29 @@
       <c r="E52" t="inlineStr">
         <is>
           <t>glenfernandes23aiml@rnsit.ac.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Demoperson</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>95</v>
+      </c>
+      <c r="D53" t="n">
+        <v>8092806977</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>demoperson011@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>